<commit_message>
Added notes - Pratik
</commit_message>
<xml_diff>
--- a/fall-2021/Attendance.xlsx
+++ b/fall-2021/Attendance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIP\Github_repos\vip-nlp\fall-2021\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D774D0A6-26AC-4C1E-B0BF-DE7542F65824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8753C0E3-851D-4E39-A130-709D817470C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -360,32 +360,30 @@
         <v>44466</v>
       </c>
       <c r="E1" s="2">
-        <v>44473</v>
+        <v>44477</v>
       </c>
       <c r="F1" s="2">
-        <v>44480</v>
+        <v>44484</v>
       </c>
       <c r="G1" s="2">
-        <v>44487</v>
+        <v>44491</v>
       </c>
       <c r="H1" s="2">
-        <v>44494</v>
+        <v>44498</v>
       </c>
       <c r="I1" s="2">
-        <v>44501</v>
+        <v>44505</v>
       </c>
       <c r="J1" s="2">
-        <v>44508</v>
+        <v>44512</v>
       </c>
       <c r="K1" s="2">
-        <v>44515</v>
+        <v>44519</v>
       </c>
       <c r="L1" s="2">
-        <v>44522</v>
-      </c>
-      <c r="M1" s="2">
         <v>44529</v>
       </c>
+      <c r="M1" s="2"/>
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
@@ -407,13 +405,13 @@
       <c r="B2" s="5"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
+      <c r="K2" s="6"/>
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
       <c r="N2" s="3"/>
@@ -440,7 +438,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="H3" s="6"/>
       <c r="I3" s="8"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -498,10 +496,10 @@
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+      <c r="F5" s="6"/>
       <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="8"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
@@ -531,7 +529,7 @@
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
-      <c r="I6" s="8"/>
+      <c r="I6" s="6"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
@@ -588,13 +586,13 @@
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="F8" s="6"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="8"/>
-      <c r="J8" s="7"/>
+      <c r="J8" s="6"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
+      <c r="L8" s="6"/>
       <c r="M8" s="7"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>

</xml_diff>